<commit_message>
script python da migliorare ma funziona!!!!!!! tutto corretto VAMOSSSSSS
</commit_message>
<xml_diff>
--- a/V5/problemGeneratorDiego/timetablingTemplateDiego.xlsx
+++ b/V5/problemGeneratorDiego/timetablingTemplateDiego.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="209" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="85">
   <si>
     <t>corso</t>
   </si>
@@ -117,9 +117,6 @@
     <t>mon12</t>
   </si>
   <si>
-    <t>mon13</t>
-  </si>
-  <si>
     <t>mon14</t>
   </si>
   <si>
@@ -306,7 +303,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -326,13 +323,6 @@
       <family val="2"/>
       <sz val="11"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <charset val="1"/>
-      <color theme="1"/>
-      <family val="1"/>
-      <sz val="10"/>
-      <name val="Times New Roman"/>
     </font>
     <font>
       <charset val="1"/>
@@ -362,7 +352,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="bottom"/>
@@ -371,9 +361,6 @@
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -699,10 +686,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BD5"/>
+  <dimension ref="A1:BC5"/>
   <sheetFormatPr defaultRowHeight="12.8" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="11.53515625" customHeight="1"/>
   <sheetData>
-    <row r="1" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="1" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -868,11 +855,8 @@
       <c r="BC1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="BD1" s="1" t="s">
-        <v>74</v>
-      </c>
     </row>
-    <row r="2" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="2" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -1038,11 +1022,8 @@
       <c r="BC2" s="1">
         <v>1</v>
       </c>
-      <c r="BD2" s="1">
-        <v>1</v>
-      </c>
     </row>
-    <row r="3" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="3" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -1208,11 +1189,8 @@
       <c r="BC3" s="1">
         <v>1</v>
       </c>
-      <c r="BD3" s="1">
-        <v>1</v>
-      </c>
     </row>
-    <row r="4" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="4" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>10</v>
       </c>
@@ -1378,16 +1356,13 @@
       <c r="BC4" s="1">
         <v>1</v>
       </c>
-      <c r="BD4" s="1">
-        <v>1</v>
-      </c>
     </row>
-    <row r="5" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="5" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C5" s="1">
         <v>0</v>
@@ -1417,7 +1392,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M5" s="1">
         <v>1</v>
@@ -1546,9 +1521,6 @@
         <v>1</v>
       </c>
       <c r="BC5" s="1">
-        <v>1</v>
-      </c>
-      <c r="BD5" s="1">
         <v>1</v>
       </c>
     </row>
@@ -1564,10 +1536,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BD4"/>
+  <dimension ref="A1:BC4"/>
   <sheetFormatPr defaultRowHeight="12.8" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="11.53515625" customHeight="1"/>
   <sheetData>
-    <row r="1" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="1" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -1733,11 +1705,8 @@
       <c r="BC1" s="1" t="s">
         <v>73</v>
       </c>
-      <c r="BD1" s="1" t="s">
-        <v>74</v>
-      </c>
     </row>
-    <row r="2" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="2" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
@@ -1772,7 +1741,7 @@
         <v>0</v>
       </c>
       <c r="L2" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M2" s="1">
         <v>1</v>
@@ -1903,11 +1872,8 @@
       <c r="BC2" s="1">
         <v>1</v>
       </c>
-      <c r="BD2" s="1">
-        <v>1</v>
-      </c>
     </row>
-    <row r="3" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="3" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>18</v>
       </c>
@@ -2073,11 +2039,8 @@
       <c r="BC3" s="1">
         <v>1</v>
       </c>
-      <c r="BD3" s="1">
-        <v>1</v>
-      </c>
     </row>
-    <row r="4" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="4" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
@@ -2241,9 +2204,6 @@
         <v>1</v>
       </c>
       <c r="BC4" s="1">
-        <v>1</v>
-      </c>
-      <c r="BD4" s="1">
         <v>1</v>
       </c>
     </row>
@@ -2264,7 +2224,7 @@
   <sheetData>
     <row r="1" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>20</v>
@@ -2427,9 +2387,6 @@
       </c>
       <c r="BC1" s="1" t="s">
         <v>73</v>
-      </c>
-      <c r="BD1" s="1" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="2" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
@@ -2467,7 +2424,7 @@
         <v>1</v>
       </c>
       <c r="L2" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M2" s="1">
         <v>0</v>
@@ -2500,7 +2457,7 @@
         <v>0</v>
       </c>
       <c r="W2" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="X2" s="1">
         <v>1</v>
@@ -2596,15 +2553,12 @@
         <v>1</v>
       </c>
       <c r="BC2" s="1">
-        <v>1</v>
-      </c>
-      <c r="BD2" s="1">
         <v>1</v>
       </c>
     </row>
     <row r="3" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B3" s="1">
         <v>1</v>
@@ -2766,9 +2720,6 @@
         <v>1</v>
       </c>
       <c r="BC3" s="1">
-        <v>1</v>
-      </c>
-      <c r="BD3" s="1">
         <v>1</v>
       </c>
     </row>
@@ -2828,11 +2779,8 @@
       <c r="BA4" s="1"/>
       <c r="BB4" s="1"/>
       <c r="BC4" s="1"/>
-      <c r="BD4" s="1"/>
     </row>
-    <row r="10" ht="13.8" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
-      <c r="G10" s="3"/>
-    </row>
+    <row r="10" ht="13.8" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -2854,45 +2802,45 @@
   <sheetData>
     <row r="1" ht="13.8" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>78</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="2" ht="13.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="B2" s="3">
+        <v>8</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>80</v>
-      </c>
-      <c r="B2" s="4">
-        <v>8</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>81</v>
       </c>
     </row>
     <row r="3" ht="13.8" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B3" s="3">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>82</v>
-      </c>
-      <c r="B3" s="4">
-        <v>0</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="D3" s="4" t="s">
-        <v>83</v>
       </c>
     </row>
     <row r="4" ht="13.8" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="5" ht="13.8" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="4" t="s">
-        <v>85</v>
+      <c r="A5" s="3" t="s">
+        <v>84</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
trovato errore pausa pranzo, da implementare. Sarebbe bello renderla dinamica e gestibile dal foglio configurazioni
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/V5/problemGeneratorDiego/timetablingTemplateDiego.xlsx
+++ b/V5/problemGeneratorDiego/timetablingTemplateDiego.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="87">
   <si>
     <t>corso</t>
   </si>
@@ -279,6 +279,16 @@
   </si>
   <si>
     <t>valori</t>
+  </si>
+  <si>
+    <r>
+      <t>ora pausa pranzo</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>13</t>
+    </r>
   </si>
   <si>
     <t>orario a costo minimo</t>
@@ -2219,10 +2229,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BD10"/>
+  <dimension ref="A1:BC10"/>
   <sheetFormatPr defaultRowHeight="12.8" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="11.53515625" customHeight="1"/>
   <sheetData>
-    <row r="1" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="1" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>75</v>
       </c>
@@ -2389,7 +2399,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="2" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>6</v>
       </c>
@@ -2556,7 +2566,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="3" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>76</v>
       </c>
@@ -2723,7 +2733,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
+    <row r="4" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -2780,7 +2790,7 @@
       <c r="BB4" s="1"/>
       <c r="BC4" s="1"/>
     </row>
-    <row r="10" ht="13.8" customHeight="1" spans="7:7" x14ac:dyDescent="0.25"/>
+    <row r="10" ht="13.8" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -2793,7 +2803,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="12.8" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="11.53515625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="40.52" style="1" customWidth="1"/>
@@ -2808,39 +2818,47 @@
         <v>78</v>
       </c>
     </row>
-    <row r="2" ht="13.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" ht="13.8" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>79</v>
       </c>
-      <c r="B2" s="3">
-        <v>8</v>
-      </c>
-      <c r="C2" s="1" t="s">
+      <c r="B2" t="s">
         <v>80</v>
       </c>
     </row>
-    <row r="3" ht="13.8" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" ht="13.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>81</v>
       </c>
       <c r="B3" s="3">
-        <v>0</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>80</v>
-      </c>
-      <c r="D3" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>82</v>
       </c>
     </row>
-    <row r="4" ht="13.8" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="4" ht="13.8" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>83</v>
       </c>
+      <c r="B4" s="3">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>84</v>
+      </c>
     </row>
     <row r="5" ht="13.8" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A5" s="3" t="s">
-        <v>84</v>
+      <c r="A5" s="1" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="6" ht="13.8" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="3" t="s">
+        <v>86</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
corretto lo script python per la generazione dei problem. TODO: grafica input (con xlsx va benissimo). grafica output importante. eventuale aggiunta costo fasce orarie
</commit_message>
<xml_diff>
--- a/V5/problemGeneratorDiego/timetablingTemplateDiego.xlsx
+++ b/V5/problemGeneratorDiego/timetablingTemplateDiego.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="86">
   <si>
     <t>corso</t>
   </si>
@@ -38,53 +38,34 @@
     <t>sistemiDigitali</t>
   </si>
   <si>
-    <r>
-      <t>sisinni</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>gruppoITID3</t>
-    </r>
+    <t>Sisinni</t>
+  </si>
+  <si>
+    <t>ITID3</t>
   </si>
   <si>
     <t>analisi</t>
   </si>
   <si>
-    <r>
-      <t>kovarik</t>
-    </r>
+    <t>Marcellini</t>
+  </si>
+  <si>
+    <t>ITID1</t>
   </si>
   <si>
     <t>componenti</t>
   </si>
   <si>
-    <r>
-      <t>bau</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>sistemiQualita</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>8</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <t>serpelloni</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-      </rPr>
-      <t>gruppoITID3</t>
-    </r>
+    <t>Bau</t>
+  </si>
+  <si>
+    <t>sistemiDiMisura</t>
+  </si>
+  <si>
+    <t>Serpelloni</t>
+  </si>
+  <si>
+    <t/>
   </si>
   <si>
     <t>aula</t>
@@ -117,6 +98,9 @@
     <t>mon12</t>
   </si>
   <si>
+    <t>mon13</t>
+  </si>
+  <si>
     <t>mon14</t>
   </si>
   <si>
@@ -264,15 +248,7 @@
     <t>fri18</t>
   </si>
   <si>
-    <t>FALSE</t>
-  </si>
-  <si>
     <t>scdla</t>
-  </si>
-  <si>
-    <r>
-      <t>gruppoInformatica3</t>
-    </r>
   </si>
   <si>
     <t>configurazioni</t>
@@ -287,7 +263,7 @@
   </si>
   <si>
     <r>
-      <t>13</t>
+      <t>12</t>
     </r>
   </si>
   <si>
@@ -325,7 +301,7 @@
       <charset val="1"/>
       <color theme="1"/>
       <family val="2"/>
-      <sz val="6"/>
+      <sz val="11"/>
       <name val="Calibri"/>
     </font>
     <font>
@@ -337,9 +313,9 @@
     <font>
       <charset val="1"/>
       <color theme="1"/>
-      <family val="2"/>
-      <sz val="11"/>
-      <name val="Calibri"/>
+      <family val="1"/>
+      <sz val="10"/>
+      <name val="Times New Roman"/>
     </font>
   </fonts>
   <fills count="2">
@@ -567,7 +543,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D5"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="12.8" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="11.53515625" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="14.93" style="1" customWidth="1"/>
@@ -615,18 +591,18 @@
         <v>8</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="4" ht="13.8" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B4" s="1">
         <v>7</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>6</v>
@@ -634,15 +610,29 @@
     </row>
     <row r="5" ht="13.8" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="B5" s="1" t="s">
         <v>12</v>
+      </c>
+      <c r="B5" s="1">
+        <v>9</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>13</v>
       </c>
       <c r="D5" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>14</v>
       </c>
     </row>
@@ -696,10 +686,10 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BC5"/>
+  <dimension ref="A1:BD5"/>
   <sheetFormatPr defaultRowHeight="12.8" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="11.53515625" customHeight="1"/>
   <sheetData>
-    <row r="1" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="1" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>2</v>
       </c>
@@ -865,8 +855,11 @@
       <c r="BC1" s="1" t="s">
         <v>73</v>
       </c>
+      <c r="BD1" s="1" t="s">
+        <v>74</v>
+      </c>
     </row>
-    <row r="2" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="2" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>5</v>
       </c>
@@ -1032,8 +1025,11 @@
       <c r="BC2" s="1">
         <v>1</v>
       </c>
+      <c r="BD2" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="3" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="3" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>8</v>
       </c>
@@ -1199,10 +1195,13 @@
       <c r="BC3" s="1">
         <v>1</v>
       </c>
+      <c r="BD3" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="4" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="4" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B4" s="1">
         <v>1</v>
@@ -1366,13 +1365,16 @@
       <c r="BC4" s="1">
         <v>1</v>
       </c>
+      <c r="BD4" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="5" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="5" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>74</v>
+      <c r="B5" s="1">
+        <v>0</v>
       </c>
       <c r="C5" s="1">
         <v>0</v>
@@ -1402,7 +1404,7 @@
         <v>0</v>
       </c>
       <c r="L5" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M5" s="1">
         <v>1</v>
@@ -1531,6 +1533,9 @@
         <v>1</v>
       </c>
       <c r="BC5" s="1">
+        <v>1</v>
+      </c>
+      <c r="BD5" s="1">
         <v>1</v>
       </c>
     </row>
@@ -1546,10 +1551,10 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BC4"/>
+  <dimension ref="A1:BD4"/>
   <sheetFormatPr defaultRowHeight="12.8" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="11.53515625" customHeight="1"/>
   <sheetData>
-    <row r="1" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="1" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>15</v>
       </c>
@@ -1715,8 +1720,11 @@
       <c r="BC1" s="1" t="s">
         <v>73</v>
       </c>
+      <c r="BD1" s="1" t="s">
+        <v>74</v>
+      </c>
     </row>
-    <row r="2" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="2" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>17</v>
       </c>
@@ -1751,7 +1759,7 @@
         <v>0</v>
       </c>
       <c r="L2" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M2" s="1">
         <v>1</v>
@@ -1882,8 +1890,11 @@
       <c r="BC2" s="1">
         <v>1</v>
       </c>
+      <c r="BD2" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="3" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="3" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>18</v>
       </c>
@@ -2049,8 +2060,11 @@
       <c r="BC3" s="1">
         <v>1</v>
       </c>
+      <c r="BD3" s="1">
+        <v>1</v>
+      </c>
     </row>
-    <row r="4" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="4" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>19</v>
       </c>
@@ -2214,6 +2228,9 @@
         <v>1</v>
       </c>
       <c r="BC4" s="1">
+        <v>1</v>
+      </c>
+      <c r="BD4" s="1">
         <v>1</v>
       </c>
     </row>
@@ -2229,10 +2246,10 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:BC10"/>
+  <dimension ref="A1:BD10"/>
   <sheetFormatPr defaultRowHeight="12.8" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="0" defaultColWidth="11.53515625" customHeight="1"/>
   <sheetData>
-    <row r="1" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="1" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>75</v>
       </c>
@@ -2398,342 +2415,351 @@
       <c r="BC1" s="1" t="s">
         <v>73</v>
       </c>
+      <c r="BD1" s="1" t="s">
+        <v>74</v>
+      </c>
     </row>
-    <row r="2" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="2" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1">
+        <v>1</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1">
+        <v>1</v>
+      </c>
+      <c r="F2" s="1">
+        <v>1</v>
+      </c>
+      <c r="G2" s="1">
+        <v>1</v>
+      </c>
+      <c r="H2" s="1">
+        <v>1</v>
+      </c>
+      <c r="I2" s="1">
+        <v>1</v>
+      </c>
+      <c r="J2" s="1">
+        <v>1</v>
+      </c>
+      <c r="K2" s="1">
+        <v>1</v>
+      </c>
+      <c r="L2" s="1">
+        <v>1</v>
+      </c>
+      <c r="M2" s="1">
+        <v>0</v>
+      </c>
+      <c r="N2" s="1">
+        <v>0</v>
+      </c>
+      <c r="O2" s="1">
+        <v>0</v>
+      </c>
+      <c r="P2" s="1">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="1">
+        <v>0</v>
+      </c>
+      <c r="R2" s="1">
+        <v>0</v>
+      </c>
+      <c r="S2" s="1">
+        <v>0</v>
+      </c>
+      <c r="T2" s="1">
+        <v>0</v>
+      </c>
+      <c r="U2" s="1">
+        <v>0</v>
+      </c>
+      <c r="V2" s="1">
+        <v>0</v>
+      </c>
+      <c r="W2" s="1">
+        <v>0</v>
+      </c>
+      <c r="X2" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y2" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AA2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AB2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AC2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AD2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AE2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AF2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AG2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AH2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AI2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AJ2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AK2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AL2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AM2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AN2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AO2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AP2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AQ2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AR2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AS2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AT2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AU2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AV2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AW2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AX2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AY2" s="1">
+        <v>1</v>
+      </c>
+      <c r="AZ2" s="1">
+        <v>1</v>
+      </c>
+      <c r="BA2" s="1">
+        <v>1</v>
+      </c>
+      <c r="BB2" s="1">
+        <v>1</v>
+      </c>
+      <c r="BC2" s="1">
+        <v>1</v>
+      </c>
+      <c r="BD2" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="1">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1">
-        <v>1</v>
-      </c>
-      <c r="D2" s="1">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1">
-        <v>1</v>
-      </c>
-      <c r="F2" s="1">
-        <v>1</v>
-      </c>
-      <c r="G2" s="1">
-        <v>1</v>
-      </c>
-      <c r="H2" s="1">
-        <v>1</v>
-      </c>
-      <c r="I2" s="1">
-        <v>1</v>
-      </c>
-      <c r="J2" s="1">
-        <v>1</v>
-      </c>
-      <c r="K2" s="1">
-        <v>1</v>
-      </c>
-      <c r="L2" s="1">
-        <v>0</v>
-      </c>
-      <c r="M2" s="1">
-        <v>0</v>
-      </c>
-      <c r="N2" s="1">
-        <v>0</v>
-      </c>
-      <c r="O2" s="1">
-        <v>0</v>
-      </c>
-      <c r="P2" s="1">
-        <v>0</v>
-      </c>
-      <c r="Q2" s="1">
-        <v>0</v>
-      </c>
-      <c r="R2" s="1">
-        <v>0</v>
-      </c>
-      <c r="S2" s="1">
-        <v>0</v>
-      </c>
-      <c r="T2" s="1">
-        <v>0</v>
-      </c>
-      <c r="U2" s="1">
-        <v>0</v>
-      </c>
-      <c r="V2" s="1">
-        <v>0</v>
-      </c>
-      <c r="W2" s="1">
-        <v>1</v>
-      </c>
-      <c r="X2" s="1">
-        <v>1</v>
-      </c>
-      <c r="Y2" s="1">
-        <v>1</v>
-      </c>
-      <c r="Z2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AA2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AB2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AC2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AD2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AE2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AF2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AG2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AH2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AI2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AJ2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AK2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AL2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AM2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AN2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AO2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AP2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AQ2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AR2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AS2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AT2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AU2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AV2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AW2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AX2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AY2" s="1">
-        <v>1</v>
-      </c>
-      <c r="AZ2" s="1">
-        <v>1</v>
-      </c>
-      <c r="BA2" s="1">
-        <v>1</v>
-      </c>
-      <c r="BB2" s="1">
-        <v>1</v>
-      </c>
-      <c r="BC2" s="1">
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1">
+        <v>1</v>
+      </c>
+      <c r="F3" s="1">
+        <v>1</v>
+      </c>
+      <c r="G3" s="1">
+        <v>1</v>
+      </c>
+      <c r="H3" s="1">
+        <v>1</v>
+      </c>
+      <c r="I3" s="1">
+        <v>1</v>
+      </c>
+      <c r="J3" s="1">
+        <v>1</v>
+      </c>
+      <c r="K3" s="1">
+        <v>1</v>
+      </c>
+      <c r="L3" s="1">
+        <v>1</v>
+      </c>
+      <c r="M3" s="1">
+        <v>1</v>
+      </c>
+      <c r="N3" s="1">
+        <v>1</v>
+      </c>
+      <c r="O3" s="1">
+        <v>1</v>
+      </c>
+      <c r="P3" s="1">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>1</v>
+      </c>
+      <c r="R3" s="1">
+        <v>1</v>
+      </c>
+      <c r="S3" s="1">
+        <v>1</v>
+      </c>
+      <c r="T3" s="1">
+        <v>1</v>
+      </c>
+      <c r="U3" s="1">
+        <v>1</v>
+      </c>
+      <c r="V3" s="1">
+        <v>1</v>
+      </c>
+      <c r="W3" s="1">
+        <v>1</v>
+      </c>
+      <c r="X3" s="1">
+        <v>1</v>
+      </c>
+      <c r="Y3" s="1">
+        <v>1</v>
+      </c>
+      <c r="Z3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AA3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AB3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AC3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AD3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AE3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AF3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AG3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AH3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AI3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AJ3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AK3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AL3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AM3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AN3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AO3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AP3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AQ3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AR3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AS3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AT3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AU3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AV3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AW3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AX3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AY3" s="1">
+        <v>1</v>
+      </c>
+      <c r="AZ3" s="1">
+        <v>1</v>
+      </c>
+      <c r="BA3" s="1">
+        <v>1</v>
+      </c>
+      <c r="BB3" s="1">
+        <v>1</v>
+      </c>
+      <c r="BC3" s="1">
+        <v>1</v>
+      </c>
+      <c r="BD3" s="1">
         <v>1</v>
       </c>
     </row>
-    <row r="3" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
-      <c r="A3" s="1" t="s">
-        <v>76</v>
-      </c>
-      <c r="B3" s="1">
-        <v>1</v>
-      </c>
-      <c r="C3" s="1">
-        <v>1</v>
-      </c>
-      <c r="D3" s="1">
-        <v>1</v>
-      </c>
-      <c r="E3" s="1">
-        <v>1</v>
-      </c>
-      <c r="F3" s="1">
-        <v>1</v>
-      </c>
-      <c r="G3" s="1">
-        <v>1</v>
-      </c>
-      <c r="H3" s="1">
-        <v>1</v>
-      </c>
-      <c r="I3" s="1">
-        <v>1</v>
-      </c>
-      <c r="J3" s="1">
-        <v>1</v>
-      </c>
-      <c r="K3" s="1">
-        <v>1</v>
-      </c>
-      <c r="L3" s="1">
-        <v>1</v>
-      </c>
-      <c r="M3" s="1">
-        <v>1</v>
-      </c>
-      <c r="N3" s="1">
-        <v>1</v>
-      </c>
-      <c r="O3" s="1">
-        <v>1</v>
-      </c>
-      <c r="P3" s="1">
-        <v>1</v>
-      </c>
-      <c r="Q3" s="1">
-        <v>1</v>
-      </c>
-      <c r="R3" s="1">
-        <v>1</v>
-      </c>
-      <c r="S3" s="1">
-        <v>1</v>
-      </c>
-      <c r="T3" s="1">
-        <v>1</v>
-      </c>
-      <c r="U3" s="1">
-        <v>1</v>
-      </c>
-      <c r="V3" s="1">
-        <v>1</v>
-      </c>
-      <c r="W3" s="1">
-        <v>1</v>
-      </c>
-      <c r="X3" s="1">
-        <v>1</v>
-      </c>
-      <c r="Y3" s="1">
-        <v>1</v>
-      </c>
-      <c r="Z3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AA3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AB3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AC3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AD3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AE3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AF3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AG3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AH3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AI3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AJ3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AK3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AL3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AM3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AN3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AO3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AP3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AQ3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AR3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AS3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AT3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AU3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AV3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AW3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AX3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AY3" s="1">
-        <v>1</v>
-      </c>
-      <c r="AZ3" s="1">
-        <v>1</v>
-      </c>
-      <c r="BA3" s="1">
-        <v>1</v>
-      </c>
-      <c r="BB3" s="1">
-        <v>1</v>
-      </c>
-      <c r="BC3" s="1">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" ht="13.8" customHeight="1" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="4" ht="13.8" customHeight="1" spans="1:56" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>
@@ -2789,8 +2815,11 @@
       <c r="BA4" s="1"/>
       <c r="BB4" s="1"/>
       <c r="BC4" s="1"/>
+      <c r="BD4" s="1"/>
     </row>
-    <row r="10" ht="13.8" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="10" ht="13.8" customHeight="1" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G10" s="3"/>
+    </row>
   </sheetData>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
@@ -2812,53 +2841,53 @@
   <sheetData>
     <row r="1" ht="13.8" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>77</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="2" ht="13.8" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="B2" t="s">
         <v>79</v>
-      </c>
-      <c r="B2" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="3" ht="13.8" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="B3" s="1">
+        <v>8</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>81</v>
-      </c>
-      <c r="B3" s="3">
-        <v>8</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="4" ht="13.8" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="B4" s="1">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>83</v>
-      </c>
-      <c r="B4" s="3">
-        <v>0</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="D4" s="3" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="5" ht="13.8" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="6" ht="13.8" customHeight="1" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A6" s="3" t="s">
-        <v>86</v>
+      <c r="A6" s="1" t="s">
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>